<commit_message>
add import frequency only
</commit_message>
<xml_diff>
--- a/public/templates/products-import-template.xlsx
+++ b/public/templates/products-import-template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>Product Name</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>SKU</t>
+  </si>
+  <si>
+    <t>frequency</t>
   </si>
 </sst>
 </file>
@@ -169,7 +172,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -192,11 +195,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -214,6 +228,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,10 +513,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC1"/>
+  <dimension ref="A1:AD1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:29" ht="65" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:30" ht="65" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -586,6 +603,9 @@
       </c>
       <c r="AC1" s="6" t="s">
         <v>25</v>
+      </c>
+      <c r="AD1" s="7" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>